<commit_message>
Fix template download on Android and edge-to-edge layout clipping
The "Download blank student sheet" link used <a download>, which Capacitor's
Android WebView doesn't wire up to anything — it silently did nothing there.
Native now fetches the file and hands it to the OS share sheet instead
(@capacitor/filesystem + @capacitor/share), so it can be saved to Drive/Files.
The served template was also missing the login_credentials tab entirely.

Separately, Android 15+ draws edge-to-edge by default, letting the system
navigation bar sit over the WebView (the attendance screen's sticky
Save & Submit bar was getting covered). MainActivity now opts back into the
classic inset behaviour so Android reserves space for system bars itself.
</commit_message>
<xml_diff>
--- a/public/templates/srm-suite-blank-template.xlsx
+++ b/public/templates/srm-suite-blank-template.xlsx
@@ -10,7 +10,8 @@
     <sheet name="children_master" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="health_and_conditions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="attendance_logs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="README" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="login_credentials" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="README" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -91,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -118,6 +119,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8756,7 +8759,54 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Password_Hash</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"viewer,editor"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9034,6 +9084,18 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>login_credentials</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Optional sign-in gate. Leave empty to skip login entirely. To add a user, open Extensions &gt; Apps Script &gt; run "setUserPassword" from the menu — it hashes the password for you, the sheet never stores it in plain text. Role is viewer (read-only) or editor (can edit records); blank = editor.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>

</xml_diff>